<commit_message>
laptop wise in image_folder_scanning
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/image_folder_insight.xlsx
+++ b/Full-LC-AUTO/image_folder_insight.xlsx
@@ -35,11 +35,11 @@
       <color rgb="001F1F1F"/>
     </font>
     <font>
+      <color rgb="007A7A7A"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00215E21"/>
-    </font>
-    <font>
-      <color rgb="007A7A7A"/>
     </font>
   </fonts>
   <fills count="8">
@@ -61,12 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -574,33 +574,33 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -611,33 +611,33 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -648,33 +648,33 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -684,34 +684,34 @@
           <t>Black-Plain</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4" t="n">
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -721,34 +721,34 @@
           <t>White-Plain</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="4" t="n">
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -758,34 +758,34 @@
           <t>Trouser</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G7" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="3" t="n">
+      <c r="H7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="K7" s="4" t="n">
         <v>9</v>
       </c>
     </row>
@@ -795,34 +795,34 @@
           <t>Shorts</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4" t="n">
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -927,28 +927,56 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Ice: missing directory -&gt; C:\work-mom\JEANS\PRODUCT IMAGES\ICE\NEW IMAGES</t>
+          <t>Black-Plain: missing directory -&gt; G:\Other computers\My Laptop\work-mom\LISTING IMAGES AUTOMATED\Black-Plain</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Black-baggy: missing directory -&gt; C:\work-mom\JEANS\PRODUCT IMAGES\BLACK-BAGGY\NEW IMAGES</t>
+          <t>Shorts: skipped folder 'Balck-Plain' (Folder name must start with a number: Balck-Plain)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Black-Plain: missing directory -&gt; C:\work-mom\JEANS\PRODUCT IMAGES\BLACK-PLAIN\NEW IMAGES</t>
+          <t>Shorts: skipped folder 'BEIGE' (Folder name must start with a number: BEIGE)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>White-Plain: missing directory -&gt; C:\work-mom\JEANS\PRODUCT IMAGES\WHITE-PLAIN\NEW IMAGES</t>
+          <t>Shorts: skipped folder 'Black-baggy' (Folder name must start with a number: Black-baggy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Shorts: skipped folder 'ICE' (Folder name must start with a number: ICE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Shorts: skipped folder 'Shorts' (Folder name must start with a number: Shorts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Shorts: skipped folder 'Trouser' (Folder name must start with a number: Trouser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Shorts: skipped folder 'White' (Folder name must start with a number: White)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AVAILABLE OPTIONS sheet in generated excel, inside image_folders_insight.py
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/image_folder_insight.xlsx
+++ b/Full-LC-AUTO/image_folder_insight.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Image Folder Insight" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Available Options" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,14 +36,14 @@
       <color rgb="001F1F1F"/>
     </font>
     <font>
-      <color rgb="007A7A7A"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00215E21"/>
     </font>
+    <font>
+      <color rgb="007A7A7A"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -61,22 +62,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE5CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDE9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -114,19 +110,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -588,8 +581,8 @@
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>0</v>
+      <c r="G2" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>0</v>
@@ -600,8 +593,8 @@
       <c r="J2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K2" s="3" t="n">
-        <v>0</v>
+      <c r="K2" s="4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -634,8 +627,8 @@
       <c r="I3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="n">
-        <v>0</v>
+      <c r="J3" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="K3" s="3" t="n">
         <v>0</v>
@@ -768,7 +761,7 @@
         <v>13</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>14</v>
@@ -837,10 +830,380 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="29" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total Numbered Folders</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Prabhu - STARVIELLE - Flipkart</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Prabhu - STARVIELLE - Shopsy</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Prabhu - GENZ VANE - Flipkart</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Prabhu - GENZ VANE - Shopsy</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Seema - FADEVIELLE - Flipkart</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Seema - FADEVIELLE - Shopsy</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Seema - FLEECRANE - Flipkart</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Seema - FLEECRANE - Shopsy</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Seema - INDIVANE - Flipkart</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Seema - INDIVANE - Shopsy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Beige</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Black-baggy</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Black-Plain</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>White-Plain</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Trouser</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Shorts</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -916,67 +1279,15 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Warnings</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Black-Plain: missing directory -&gt; G:\Other computers\My Laptop\work-mom\LISTING IMAGES AUTOMATED\Black-Plain</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'Balck-Plain' (Folder name must start with a number: Balck-Plain)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'BEIGE' (Folder name must start with a number: BEIGE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'Black-baggy' (Folder name must start with a number: Black-baggy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'ICE' (Folder name must start with a number: ICE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'Shorts' (Folder name must start with a number: Shorts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'Trouser' (Folder name must start with a number: Trouser)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Shorts: skipped folder 'White' (Folder name must start with a number: White)</t>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Available Options</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Each value is total numbered folders minus exhausted count for that account/brand/surface</t>
         </is>
       </c>
     </row>

</xml_diff>